<commit_message>
fix(F-NAR-008): leçon implicite (ranger, règle, rire, colère)
Le doudou se retrouve sous le bazar. On ne dit plus « on va ranger »
ni « c'est la règle » ni « même leçon ».
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-02.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-02.xlsx
@@ -1953,12 +1953,12 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les deux filles se tiennent la main. Le linge fait une ombre sur le sol. On est dans la cour. Oui, tu es arrivée. Le sac vert repose près du pot. L'orange de la cuisine sent encore. Bravo, tu as préparé tout ça. Le linge blanc sèche encore, tout calme.</t>
+          <t>Les deux filles se tiennent la main. Le linge fait une ombre sur le sol. On est dans la cour. Oui, tu es arrivée. Le sac vert repose près du pot. L'orange de la cuisine sent encore. Le doudou est chaud, dans le sac. Le linge blanc sèche encore, tout calme.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les deux filles se tiennent la main. Le linge fait une ombre sur le sol. On est dans la cour. Oui, tu es arrivée. Le sac vert repose près du pot. L'orange de la cuisine sent encore. Bravo, tu as préparé tout ça. Le linge blanc sèche encore, tout calme.</t>
+          <t>Les deux filles se tiennent la main. Le linge fait une ombre sur le sol. On est dans la cour. Oui, tu es arrivée. Le sac vert repose près du pot. L'orange de la cuisine sent encore. Le doudou est chaud, dans le sac. Le linge blanc sèche encore, tout calme.</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
 maman|Oui, tu es arrivée.
 narrateur|Le sac vert repose près du pot.
 narrateur|L'orange de la cuisine sent encore.
-maman|Bravo, tu as préparé tout ça.
+maman|Le doudou est chaud, dans le sac.
 narrateur|Le linge blanc sèche encore, tout calme.</t>
         </is>
       </c>
@@ -2121,7 +2121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2178,6 +2178,13 @@
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): ATOM-AUT.AFF.001-02 La cour de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-02.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-02.xlsx
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sarah veut retrouver Chouchou dans la cour de l'immeuble. Le chapeau est sous la chaise, la sangle coincée. Elle range, descend. Le linge danse pour elles.</t>
+          <t>Sarah veut pincer sa serviette bleue sur le fil de la cour, maintenant. Un éclat de pince saute sur la table. Elle bourre le sac trop vite, le zip refuse. Elle arrête de forcer, range, descend. Chouchou tire vers le chat ; Sarah refuse de foncer, retrouve l'éclat, pince le tissu. Le sac repose près du pot fêlé.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Dans la cour, un linge blanc sèche. Il claque un peu contre le fil. Les marches de l'immeuble sentent le savon. Une plante verte pousse dans un pot. Le pot est fêlé, tout doux au bord. Un chat gris passe dans l'ombre. La cage d'escalier est un peu fraîche. Au troisième, la porte de Sarah est ouverte. La cuisine sent l'orange pressée. Sarah, tu as vu le linge ? Oui, maman. Il danse. Chouchou t'attend en bas. Je veux la voir. On descend, avec le sac. En ce moment, Sarah prend le sac vert. Le tissu est un peu rêche. Il est vert, maman. Oui, c'est le tien. Mets de l'eau, pour la cour. Sarah prend la gourde. Elle est fraîche contre ses doigts. Sarah la glisse dans le sac. Ton chapeau aussi, le soleil tape. Sarah cherche près de la chaise. La chaise est vide. Il n'est pas là. Regarde sous le siège. Le chapeau souple est par terre. Sarah le plie tout doucement. Elle le pose dans le sac. Et mon doudou ? Il voudra Chouchou aussi. Le doudou gris a les oreilles plates. Il sent encore l'oreiller. Sarah le serre, puis le glisse. La sangle se coince dans le zip. Ça reste, maman. Doucement, tu peux l'aider.</t>
+          <t>Un clac monte l'escalier de pierre. C'est le drap, en bas, sur le fil. Sarah connaît cette cour. En bas, un pot est fêlé. Une plante verte y pousse. Les marches sentent le savon. Au troisième, la fenêtre est ouverte. La cuisine sent l'orange pressée. Un éclat saute sur la table. Ce n'est pas le jus. C'est un éclat de pince. La pince tient le drap, en bas. Sarah, tu as vu le linge ? Oui, maman. Il danse. Chouchou t'attend près du pot. Je veux descendre maintenant ! On prend le sac, d'abord. En ce moment, Sarah saisit le sac vert. Le tissu gratte sous ses doigts. Il est à moi. Oui, c'est le tien. Près du sac, une serviette bleue. Elle est un peu humide. Je veux la pincer, là-bas ! Mets l'eau, pour la cour. Sarah pousse la gourde d'un coup. La gourde bascule contre le tissu. Vite, maman ! Ton chapeau aussi, le soleil tape. Sarah cherche près de la chaise. La chaise est vide. Il n'est pas là. Le chapeau souple est par terre. Elle le jette dans le sac. Et mon doudou ? Il voudra voir Chouchou. Le doudou gris a les oreilles plates. Il sent l'oreiller de la chambre. Sarah le glisse, trop vite. La sangle se coince dans le zip. Ça reste, maman ! Elle tire plus fort. Le zip refuse. Le sourire de Sarah disparaît. Dans sa poitrine, ça se bouscule. Maman s'accroupit à la même hauteur. Tu veux forcer, ou regarder ? Je veux Chouchou. Sarah tire une dernière fois. Rien ne bouge. Elle baisse les épaules.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Dans la cour, un linge blanc sèche. Il claque un peu contre le fil. Les marches de l'immeuble sentent le savon. Une plante verte pousse dans un pot. Le pot est fêlé, tout doux au bord. Un chat gris passe dans l'ombre. La cage d'escalier est un peu fraîche. Au troisième, la porte de Sarah est ouverte. La cuisine sent l'orange pressée. Sarah, tu as vu le linge ? Oui, maman. Il danse. Chouchou t'attend en bas. Je veux la voir. On descend, avec le sac. En ce moment, Sarah prend le sac vert. Le tissu est un peu rêche. Il est vert, maman. Oui, c'est le tien. Mets de l'eau, pour la cour. Sarah prend la gourde. Elle est fraîche contre ses doigts. Sarah la glisse dans le sac. Ton chapeau aussi, le soleil tape. Sarah cherche près de la chaise. La chaise est vide. Il n'est pas là. Regarde sous le siège. Le chapeau souple est par terre. Sarah le plie tout doucement. Elle le pose dans le sac. Et mon doudou ? Il voudra Chouchou aussi. Le doudou gris a les oreilles plates. Il sent encore l'oreiller. Sarah le serre, puis le glisse. La sangle se coince dans le zip. Ça reste, maman. Doucement, tu peux l'aider.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Un clac monte l'escalier de pierre. C'est le drap, en bas, sur le fil. Sarah connaît cette cour. En bas, un pot est fêlé. Une plante verte y pousse. Les marches sentent le savon. Au troisième, la fenêtre est ouverte. La cuisine sent l'orange pressée. Un éclat saute sur la table. Ce n'est pas le jus. C'est un &lt;emphasis level="moderate"&gt;éclat de pince&lt;/emphasis&gt;. La pince tient le drap, en bas. Sarah, tu as vu le linge ? Oui, maman. Il danse. Chouchou t'attend près du pot. Je veux descendre maintenant ! On prend le sac, d'abord. En ce moment, Sarah saisit le sac vert. Le tissu gratte sous ses doigts. Il est à moi. Oui, c'est le tien. Près du sac, une serviette bleue. Elle est un peu humide. Je veux la pincer, là-bas ! Mets l'eau, pour la cour. Sarah pousse la gourde d'un coup. La gourde bascule contre le tissu. Vite, maman ! Ton chapeau aussi, le soleil tape. Sarah cherche près de la chaise. La chaise est vide. Il n'est pas là. Le chapeau souple est par terre. Elle le jette dans le sac. Et mon doudou ? Il voudra voir Chouchou. Le doudou gris a les oreilles plates. Il sent l'oreiller de la chambre. Sarah le glisse, trop vite. La sangle se coince dans le zip. Ça reste, maman ! Elle tire plus fort. Le zip refuse. Le sourire de Sarah disparaît. Dans sa poitrine, ça se bouscule. Maman s'accroupit à la même hauteur. Tu veux forcer, ou regarder ? Je veux Chouchou. Sarah tire une dernière fois. Rien ne bouge. Elle baisse les épaules.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Iris est dans sa chambre. Le &lt;emphasis&gt;sac&lt;/emphasis&gt; est sur le lit. Il est vert. Maman est là. Maman est l'adulte. Maman dit : le chapeau, le doudou, la gourde. Iris écoute. Elle voit le chapeau. Elle le met dans le sac. Elle voit le doudou doux. Elle le met dans le sac. Elle voit la gourde. Elle la met dans le sac. Iris appuie sur la fermeture. Ça fait zzz. Iris a mis ce que l'adulte a dit. Maman dit : merci Iris. Le sac est prêt.&lt;/slow&gt; [pause]</t>
+          <t>Un clac monte l'escalier de pierre. C'est le drap, en bas, sur le fil. Sarah connaît cette cour. En bas, un pot est fêlé. Une plante verte y pousse. Les marches sentent le savon. Au troisième, la fenêtre est ouverte. La cuisine sent l'orange pressée. Un éclat saute sur la table. Ce n'est pas le jus. C'est un &lt;emphasis&gt;éclat de pince&lt;/emphasis&gt;. La pince tient le drap, en bas. Sarah, tu as vu le linge ? Oui, maman. Il danse. Chouchou t'attend près du pot. Je veux descendre maintenant ! On prend le sac, d'abord. En ce moment, Sarah saisit le sac vert. Le tissu gratte sous ses doigts. Il est à moi. Oui, c'est le tien. Près du sac, une serviette bleue. Elle est un peu humide. Je veux la pincer, là-bas ! Mets l'eau, pour la cour. Sarah pousse la gourde d'un coup. La gourde bascule contre le tissu. Vite, maman ! Ton chapeau aussi, le soleil tape. Sarah cherche près de la chaise. La chaise est vide. Il n'est pas là. Le chapeau souple est par terre. Elle le jette dans le sac. Et mon doudou ? Il voudra voir Chouchou. Le doudou gris a les oreilles plates. Il sent l'oreiller de la chambre. Sarah le glisse, trop vite. La sangle se coince dans le zip. Ça reste, maman ! Elle tire plus fort. Le zip refuse. Le sourire de Sarah disparaît. Dans sa poitrine, ça se bouscule. Maman s'accroupit à la même hauteur. Tu veux forcer, ou regarder ? Je veux Chouchou. Sarah tire une dernière fois. Rien ne bouge. Elle baisse les épaules. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.22</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de pince</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,50 +1319,72 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller; emotion=impatience_curieuse; intensite=2; destinataire=enfant; sous_texte=l_eclat_de_pince_saute_sur_la_table; tempo=naturel; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Dans la cour, un linge blanc sèche.
-narrateur|Il claque un peu contre le fil.
-narrateur|Les marches de l'immeuble sentent le savon.
-narrateur|Une plante verte pousse dans un pot.
-narrateur|Le pot est fêlé, tout doux au bord.
-narrateur|Un chat gris passe dans l'ombre.
-narrateur|La cage d'escalier est un peu fraîche.
-narrateur|Au troisième, la porte de Sarah est ouverte.
+          <t>narrateur|Un clac monte l'escalier de pierre.
+narrateur|C'est le drap, en bas, sur le fil.
+narrateur|Sarah connaît cette cour.
+narrateur|En bas, un pot est fêlé.
+narrateur|Une plante verte y pousse.
+narrateur|Les marches sentent le savon.
+narrateur|Au troisième, la fenêtre est ouverte.
 narrateur|La cuisine sent l'orange pressée.
+narrateur|Un éclat saute sur la table.
+narrateur|Ce n'est pas le jus.
+narrateur|C'est un éclat de pince.
+narrateur|La pince tient le drap, en bas.
 maman|Sarah, tu as vu le linge ?
 enfant-f|Oui, maman.
 enfant-f|Il danse.
-maman|Chouchou t'attend en bas.
-enfant-f|Je veux la voir.
-maman|On descend, avec le sac.
-narrateur|En ce moment, Sarah prend le sac vert.
-narrateur|Le tissu est un peu rêche.
-enfant-f|Il est vert, maman.
+maman|Chouchou t'attend près du pot.
+enfant-f|Je veux descendre maintenant !
+maman|On prend le sac, d'abord.
+narrateur|En ce moment, Sarah saisit le sac vert.
+narrateur|Le tissu gratte sous ses doigts.
+enfant-f|Il est à moi.
 maman|Oui, c'est le tien.
-maman|Mets de l'eau, pour la cour.
-narrateur|Sarah prend la gourde.
-narrateur|Elle est fraîche contre ses doigts.
-narrateur|Sarah la glisse dans le sac.
+narrateur|Près du sac, une serviette bleue.
+narrateur|Elle est un peu humide.
+enfant-f|Je veux la pincer, là-bas !
+maman|Mets l'eau, pour la cour.
+narrateur|Sarah pousse la gourde d'un coup.
+narrateur|La gourde bascule contre le tissu.
+enfant-f|Vite, maman !
 maman|Ton chapeau aussi, le soleil tape.
 narrateur|Sarah cherche près de la chaise.
 narrateur|La chaise est vide.
 enfant-f|Il n'est pas là.
-maman|Regarde sous le siège.
 narrateur|Le chapeau souple est par terre.
-narrateur|Sarah le plie tout doucement.
-narrateur|Elle le pose dans le sac.
+narrateur|Elle le jette dans le sac.
 enfant-f|Et mon doudou ?
-maman|Il voudra Chouchou aussi.
+maman|Il voudra voir Chouchou.
 narrateur|Le doudou gris a les oreilles plates.
-narrateur|Il sent encore l'oreiller.
-narrateur|Sarah le serre, puis le glisse.
+narrateur|Il sent l'oreiller de la chambre.
+narrateur|Sarah le glisse, trop vite.
 narrateur|La sangle se coince dans le zip.
-enfant-f|Ça reste, maman.
-maman|Doucement, tu peux l'aider.</t>
+enfant-f|Ça reste, maman !
+narrateur|Elle tire plus fort.
+narrateur|Le zip refuse.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|Maman s'accroupit à la même hauteur.
+maman|Tu veux forcer, ou regarder ?
+enfant-f|Je veux Chouchou.
+narrateur|Sarah tire une dernière fois.
+narrateur|Rien ne bouge.
+narrateur|Elle baisse les épaules.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>linge,savon</t>
         </is>
       </c>
     </row>
@@ -1389,17 +1411,17 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Sarah prépare le sac. Où met-elle les affaires ?</t>
+          <t>Sarah prépare le sac pour descendre. Où met-elle les affaires ?</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sarah prépare le sac. Où met-elle les affaires ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Sarah prépare le &lt;emphasis level="moderate"&gt;sac&lt;/emphasis&gt; pour descendre. Où met-elle les affaires ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Iris prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Que fait-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Sarah prépare le &lt;emphasis&gt;sac&lt;/emphasis&gt; pour descendre. Où met-elle les affaires ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1462,7 +1484,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1470,10 +1492,10 @@
         </is>
       </c>
       <c r="AA3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.28</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1488,11 +1510,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1503,23 +1525,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1528,13 +1550,13 @@
         </is>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1544,13 +1566,13 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=les_affaires_vont_dans_le_sac; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
         <is>
-          <t>narrateur|Sarah prépare le sac.
-narrateur|Où met-elle les affaires ?</t>
+          <t>narrateur|Sarah prépare le sac pour descendre.
+maman|Où met-elle les affaires ?</t>
         </is>
       </c>
     </row>
@@ -1577,17 +1599,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah pince le tissu coincé. Elle le tire vers elle, tout bas. Le zip avance, petit à petit. Il part. Merci, Sarah. Tu l'as aidé. Sarah appuie encore un peu. Ça fait zzz, tout doux. Le sac vert est fermé. Le sac est prêt ? Oui, maman. Sarah pose le sac contre sa jambe. Le vert brille un peu. Le cheval de bois reste sur le lit. Le cheval reste ici. Le doudou vient. On descend voir Chouchou ? Oui.</t>
+          <t>J'arrête de tirer. Elle lâche le zip. Un fil du sac brille un peu. Comme la pince. Sarah pince le tissu coincé. Elle le tire vers elle, sans forcer. Le zip avance, petit à petit. Il part ! Tu l'as aidé, toi. Sarah glisse le chapeau, sans jeter. Toi aussi, gourde. La gourde rentre, bien droite. Le doudou glisse près de l'eau. Vous êtes dedans. Tu fermes, maintenant ? Sarah appuie sur la fermeture. Ça fait zzz, très bas. Le sac vert est fermé. Le sac est prêt ? Oui, maman. Sarah pose le sac contre sa jambe. Le vert brille un peu. On descend voir Chouchou ? Oui.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah pince le tissu coincé. Elle le tire vers elle, tout bas. Le zip avance, petit à petit. Il part. Merci, Sarah. Tu l'as aidé. Sarah appuie encore un peu. Ça fait zzz, tout doux. Le sac vert est fermé. Le sac est prêt ? Oui, maman. Sarah pose le sac contre sa jambe. Le vert brille un peu. Le cheval de bois reste sur le lit. Le cheval reste ici. Le doudou vient. On descend voir Chouchou ? Oui.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;J'arrête de tirer. Elle lâche le &lt;emphasis level="moderate"&gt;zip&lt;/emphasis&gt;. Un fil du sac brille un peu. Comme la pince. Sarah pince le tissu coincé. Elle le tire vers elle, sans forcer. Le zip avance, petit à petit. Il part ! Tu l'as aidé, toi. Sarah glisse le chapeau, sans jeter. Toi aussi, gourde. La gourde rentre, bien droite. Le doudou glisse près de l'eau. Vous êtes dedans. Tu fermes, maintenant ? Sarah appuie sur la fermeture. Ça fait zzz, très bas. Le sac vert est fermé. Le sac est prêt ? Oui, maman. Sarah pose le sac contre sa jambe. Le vert brille un peu. On descend voir Chouchou ? Oui.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Iris a préparé le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Elle a mis ce que l'adulte a dit. Maman était là.&lt;/slow&gt; [pause]</t>
+          <t>J'arrête de tirer. Elle lâche le &lt;emphasis&gt;zip&lt;/emphasis&gt;. Un fil du sac brille un peu. Comme la pince. Sarah pince le tissu coincé. Elle le tire vers elle, sans forcer. Le zip avance, petit à petit. Il part ! Tu l'as aidé, toi. Sarah glisse le chapeau, sans jeter. Toi aussi, gourde. La gourde rentre, bien droite. Le doudou glisse près de l'eau. Vous êtes dedans. Tu fermes, maintenant ? Sarah appuie sur la fermeture. Ça fait zzz, très bas. Le sac vert est fermé. Le sac est prêt ? Oui, maman. Sarah pose le sac contre sa jambe. Le vert brille un peu. On descend voir Chouchou ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1634,7 +1656,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1642,10 +1664,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.22</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1668,30 +1690,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>zip</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1700,10 +1722,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1712,35 +1734,46 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_la_réussite; emotion=fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_cesse_de_forcer_le_zip_part; tempo=naturel; sourire=franc; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah pince le tissu coincé.
-narrateur|Elle le tire vers elle, tout bas.
+          <t>enfant-f|J'arrête de tirer.
+narrateur|Elle lâche le zip.
+narrateur|Un fil du sac brille un peu.
+enfant-f|Comme la pince.
+narrateur|Sarah pince le tissu coincé.
+narrateur|Elle le tire vers elle, sans forcer.
 narrateur|Le zip avance, petit à petit.
-enfant-f|Il part.
-maman|Merci, Sarah.
-maman|Tu l'as aidé.
-narrateur|Sarah appuie encore un peu.
-narrateur|Ça fait zzz, tout doux.
+enfant-f|Il part !
+maman|Tu l'as aidé, toi.
+narrateur|Sarah glisse le chapeau, sans jeter.
+enfant-f|Toi aussi, gourde.
+narrateur|La gourde rentre, bien droite.
+narrateur|Le doudou glisse près de l'eau.
+enfant-f|Vous êtes dedans.
+maman|Tu fermes, maintenant ?
+narrateur|Sarah appuie sur la fermeture.
+narrateur|Ça fait zzz, très bas.
 narrateur|Le sac vert est fermé.
 maman|Le sac est prêt ?
 enfant-f|Oui, maman.
 narrateur|Sarah pose le sac contre sa jambe.
 narrateur|Le vert brille un peu.
-narrateur|Le cheval de bois reste sur le lit.
-maman|Le cheval reste ici.
-enfant-f|Le doudou vient.
 maman|On descend voir Chouchou ?
 enfant-f|Oui.</t>
         </is>
       </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>zip</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -1765,17 +1798,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Les marches sont un peu froides. Un voisin ferme une porte, tout loin. Elles arrivent dans la cour. Le linge blanc claque encore. Chouchou est près du pot fêlé. Je suis là ! Elle t'attendait. Sarah s'accroupit près du pot. La terre du pot est un peu sèche. Le linge danse, tu vois ? Oui, pour vous deux. Un chat gris revient dans l'ombre. Sarah ouvre un tout petit peu le sac. Doudou, tu vois Chouchou ? Il la voit, dedans.</t>
+          <t>Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Les marches sont un peu froides. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'éclat de pince est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Les marches sont un peu froides. Un voisin ferme une porte, tout loin. Elles arrivent dans la cour. Le linge blanc claque encore. Chouchou est près du pot fêlé. Je suis là ! Elle t'attendait. Sarah s'accroupit près du pot. La terre du pot est un peu sèche. Le linge danse, tu vois ? Oui, pour vous deux. Un chat gris revient dans l'ombre. Sarah ouvre un tout petit peu le sac. Doudou, tu vois Chouchou ? Il la voit, dedans.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Les marches sont un peu froides. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'&lt;emphasis level="moderate"&gt;éclat de pince&lt;/emphasis&gt; est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Iris porte le &lt;emphasis&gt;sac&lt;/emphasis&gt;. Maman ouvre la porte.&lt;/slow&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Les marches sont un peu froides. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'&lt;emphasis&gt;éclat de pince&lt;/emphasis&gt; est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1822,7 +1855,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1830,22 +1863,26 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.22</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="AD5" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="AE5" s="2" t="inlineStr"/>
+          <t>-2st</t>
+        </is>
+      </c>
+      <c r="AE5" s="2" t="inlineStr">
+        <is>
+          <t>low-pitch</t>
+        </is>
+      </c>
       <c r="AF5" s="2" t="inlineStr">
         <is>
           <t>medium</t>
@@ -1856,30 +1893,30 @@
       </c>
       <c r="AH5" s="2" t="inlineStr">
         <is>
-          <t>sac</t>
+          <t>éclat de pince</t>
         </is>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>520</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>tense</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1888,21 +1925,25 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=obstacle; intention=alerter_sans_effrayer; emotion=deux_envies_qui_se_heurtent; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_retrouve_l_eclat; tempo=resserré; sourire=aucun; respiration=retenue</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
           <t>narrateur|Sarah porte le sac.
@@ -1912,21 +1953,38 @@
 narrateur|La cage d'escalier sent le savon.
 maman|Tu as ton sac ?
 enfant-f|Oui, maman.
+narrateur|Un pas, puis un autre.
+narrateur|La rampe est lisse, un peu froide.
 narrateur|Les marches sont un peu froides.
-narrateur|Un voisin ferme une porte, tout loin.
-narrateur|Elles arrivent dans la cour.
-narrateur|Le linge blanc claque encore.
+narrateur|Un voisin ferme une porte, loin.
+narrateur|La cour s'ouvre, claire.
+narrateur|Le drap blanc claque sur le fil.
 narrateur|Chouchou est près du pot fêlé.
 enfant-f|Je suis là !
-maman|Elle t'attendait.
-narrateur|Sarah s'accroupit près du pot.
-narrateur|La terre du pot est un peu sèche.
-enfant-f|Le linge danse, tu vois ?
-maman|Oui, pour vous deux.
-narrateur|Un chat gris revient dans l'ombre.
-narrateur|Sarah ouvre un tout petit peu le sac.
-enfant-f|Doudou, tu vois Chouchou ?
-maman|Il la voit, dedans.</t>
+narrateur|Chouchou court vers Sarah.
+enfant-f|Viens, le chat part !
+narrateur|Sarah veut accrocher sa serviette.
+narrateur|Les deux envies se heurtent.
+narrateur|Sarah s'arrête net.
+enfant-f|Pas maintenant.
+narrateur|Elle refuse de foncer.
+narrateur|Elle lève les yeux vers le fil.
+narrateur|L'éclat de pince est là.
+narrateur|Celui de la table, ce matin.
+enfant-f|D'abord le fil.
+narrateur|Elle sort la serviette bleue.
+maman|Tu veux une pince ?
+enfant-f|Celle qui brille.
+narrateur|Sarah pose le tissu près du drap.
+narrateur|Elle pince, sans se presser.
+narrateur|La serviette tient.
+narrateur|Chouchou s'approche du fil.
+enfant-f|Ça brille !</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>pas,linge</t>
         </is>
       </c>
     </row>
@@ -1953,17 +2011,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Les deux filles se tiennent la main. Le linge fait une ombre sur le sol. On est dans la cour. Oui, tu es arrivée. Le sac vert repose près du pot. L'orange de la cuisine sent encore. Le doudou est chaud, dans le sac. Le linge blanc sèche encore, tout calme.</t>
+          <t>Les deux filles regardent le fil. La serviette bleue danse un peu. L'éclat de pince reste sur le métal. Le sac vert repose près du pot. Merci d'avoir regardé, Sarah. Tu as vu la pince, toi ? Elle m'a montré le fil. Le doudou est au chaud, dans le sac. Le drap blanc fait une ombre ronde. Un chat gris passe dans l'ombre. On est dans la cour. Oui, vous y êtes. Elles se tiennent la main.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Les deux filles se tiennent la main. Le linge fait une ombre sur le sol. On est dans la cour. Oui, tu es arrivée. Le sac vert repose près du pot. L'orange de la cuisine sent encore. Le doudou est chaud, dans le sac. Le linge blanc sèche encore, tout calme.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les deux filles regardent le fil. La serviette bleue danse un peu. L'&lt;emphasis level="moderate"&gt;éclat de pince&lt;/emphasis&gt; reste sur le métal. Le sac vert repose près du pot. Merci d'avoir regardé, Sarah. Tu as vu la pince, toi ? Elle m'a montré le fil. Le doudou est au chaud, dans le sac. Le drap blanc fait une ombre ronde. Un chat gris passe dans l'ombre. On est dans la cour. Oui, vous y êtes. Elles se tiennent la main.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les deux filles regardent le fil. La serviette bleue danse un peu. L'&lt;emphasis&gt;éclat de pince&lt;/emphasis&gt; reste sur le métal. Le sac vert repose près du pot. Merci d'avoir regardé, Sarah. Tu as vu la pince, toi ? Elle m'a montré le fil. Le doudou est au chaud, dans le sac. Le drap blanc fait une ombre ronde. Un chat gris passe dans l'ombre. On est dans la cour. Oui, vous y êtes. Elles se tiennent la main.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2010,18 +2068,18 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>slow</t>
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.22</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2030,12 +2088,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2044,17 +2102,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de pince</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>380</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2063,11 +2125,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2076,31 +2138,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_de_pince_paie_le_debut; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|Les deux filles se tiennent la main.
-narrateur|Le linge fait une ombre sur le sol.
+          <t>narrateur|Les deux filles regardent le fil.
+narrateur|La serviette bleue danse un peu.
+narrateur|L'éclat de pince reste sur le métal.
+narrateur|Le sac vert repose près du pot.
+maman|Merci d'avoir regardé, Sarah.
+maman|Tu as vu la pince, toi ?
+enfant-f|Elle m'a montré le fil.
+narrateur|Le doudou est au chaud, dans le sac.
+narrateur|Le drap blanc fait une ombre ronde.
+narrateur|Un chat gris passe dans l'ombre.
 enfant-f|On est dans la cour.
-maman|Oui, tu es arrivée.
-narrateur|Le sac vert repose près du pot.
-narrateur|L'orange de la cuisine sent encore.
-maman|Le doudou est chaud, dans le sac.
-narrateur|Le linge blanc sèche encore, tout calme.</t>
+maman|Oui, vous y êtes.
+narrateur|Elles se tiennent la main.</t>
+        </is>
+      </c>
+      <c r="AX6" t="inlineStr">
+        <is>
+          <t>linge</t>
         </is>
       </c>
     </row>
@@ -2121,7 +2197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2185,6 +2261,13 @@
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>

<commit_message>
feat(F-NAR-019): polish ATOM-AUT.AFF.001-02 xlsx
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-AUT.AFF.001-02.xlsx
+++ b/stories/arbres/ATOM-AUT.AFF.001-02.xlsx
@@ -1798,17 +1798,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Les marches sont un peu froides. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'éclat de pince est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !</t>
+          <t>Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Tu tiens la rampe ? Oui. Les marches piquent un peu les pieds. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Sarah lève la main. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'éclat de pince est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Les marches sont un peu froides. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'&lt;emphasis level="moderate"&gt;éclat de pince&lt;/emphasis&gt; est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Tu tiens la rampe ? Oui. Les marches piquent un peu les pieds. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Sarah lève la main. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'&lt;emphasis level="moderate"&gt;éclat de pince&lt;/emphasis&gt; est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Les marches sont un peu froides. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'&lt;emphasis&gt;éclat de pince&lt;/emphasis&gt; est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Sarah porte le sac. Les bretelles sont souples. On va vers la porte. Elles quittent l'appartement. La cage d'escalier sent le savon. Tu as ton sac ? Oui, maman. Un pas, puis un autre. La rampe est lisse, un peu froide. Tu tiens la rampe ? Oui. Les marches piquent un peu les pieds. Un voisin ferme une porte, loin. La cour s'ouvre, claire. Le drap blanc claque sur le fil. Chouchou est près du pot fêlé. Sarah lève la main. Je suis là ! Chouchou court vers Sarah. Viens, le chat part ! Sarah veut accrocher sa serviette. Les deux envies se heurtent. Sarah s'arrête net. Pas maintenant. Elle refuse de foncer. Elle lève les yeux vers le fil. L'&lt;emphasis&gt;éclat de pince&lt;/emphasis&gt; est là. Celui de la table, ce matin. D'abord le fil. Elle sort la serviette bleue. Tu veux une pince ? Celle qui brille. Sarah pose le tissu près du drap. Elle pince, sans se presser. La serviette tient. Chouchou s'approche du fil. Ça brille !&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1955,11 +1955,14 @@
 enfant-f|Oui, maman.
 narrateur|Un pas, puis un autre.
 narrateur|La rampe est lisse, un peu froide.
-narrateur|Les marches sont un peu froides.
+maman|Tu tiens la rampe ?
+enfant-f|Oui.
+narrateur|Les marches piquent un peu les pieds.
 narrateur|Un voisin ferme une porte, loin.
 narrateur|La cour s'ouvre, claire.
 narrateur|Le drap blanc claque sur le fil.
 narrateur|Chouchou est près du pot fêlé.
+narrateur|Sarah lève la main.
 enfant-f|Je suis là !
 narrateur|Chouchou court vers Sarah.
 enfant-f|Viens, le chat part !
@@ -2197,7 +2200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2268,6 +2271,13 @@
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>